<commit_message>
merged sam and olivia's segments of the proposal, formatted it
</commit_message>
<xml_diff>
--- a/Research Logs/Matt/Matt Baker - Week 4 Research Log.xlsx
+++ b/Research Logs/Matt/Matt Baker - Week 4 Research Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\Weltec\IT 7510 Capstone\Week 4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Research Logs\Matt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C505BA06-6501-4143-ABEA-D918B249A916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9108FB-8F29-4FB8-900A-DDA0996028AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>Date</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>Listened to a podcast where forensic examiner with 24 year's experience Heather Barngarter goes over the philosophy behind a framework for determining where and where not AI has a place in DFIR, the prevailing sentiment is that it does not belong in digital forensics, but could be useful in incident response. AI can be used to "find a thread to pull" or to discover something in a case previously unseen, but the risks are too great due to unvalidatable results, lack of accountability when something goes wrong, the inability to resolve insights that are not there and much more, it is a tool, a tool does not determine guilt, the forensic examiner and investigator does.</t>
+  </si>
+  <si>
+    <t>WEEK 4</t>
   </si>
 </sst>
 </file>
@@ -536,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G18"/>
+  <dimension ref="B2:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.140625" style="3" customWidth="1"/>
@@ -552,7 +555,7 @@
         <v>3</v>
       </c>
       <c r="D2" s="5">
-        <f>ROUNDDOWN(SUM(C6:C500)/60,0)</f>
+        <f>ROUNDDOWN(SUM(C6:C499)/60,0)</f>
         <v>4</v>
       </c>
       <c r="E2" t="s">
@@ -564,7 +567,7 @@
         <v>4</v>
       </c>
       <c r="D3" s="5">
-        <f>ROUND(MOD(SUM(C6:C500),60),0)</f>
+        <f>ROUND(MOD(SUM(C6:C499),60),0)</f>
         <v>45</v>
       </c>
     </row>
@@ -688,6 +691,11 @@
         <v>25</v>
       </c>
     </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
     <row r="13" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <v>46239</v>
@@ -708,7 +716,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" ht="105" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <v>46239</v>
       </c>
@@ -721,66 +729,64 @@
       <c r="E14" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="2:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="F14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="B15" s="3">
+        <v>46239</v>
+      </c>
+      <c r="C15">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" t="s">
+        <v>27</v>
+      </c>
       <c r="F15" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" ht="90" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="195" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <v>46239</v>
       </c>
       <c r="C16">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E16" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" ht="195" x14ac:dyDescent="0.25">
-      <c r="B17" s="3">
-        <v>46239</v>
-      </c>
-      <c r="C17">
-        <v>60</v>
-      </c>
-      <c r="D17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" t="s">
-        <v>35</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G17" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F18" s="1"/>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F17" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G8" r:id="rId1" xr:uid="{2D576095-DD33-41E2-AE3D-624BFE4181D0}"/>
     <hyperlink ref="G9" r:id="rId2" xr:uid="{4C5458C7-3251-4B50-B993-29D9C5092585}"/>
     <hyperlink ref="G10" r:id="rId3" xr:uid="{37D06B73-17A9-4592-98F1-C038CB44CDA2}"/>
-    <hyperlink ref="G16" r:id="rId4" xr:uid="{AAFD389F-5339-488C-8F44-9A3F039DCFDD}"/>
-    <hyperlink ref="G17" r:id="rId5" display="https://open.spotify.com/episode/6Rljo1PtpUiz0N779Muyp0" xr:uid="{174DB1DB-772B-43EC-AFB0-0428427A70E8}"/>
+    <hyperlink ref="G15" r:id="rId4" xr:uid="{AAFD389F-5339-488C-8F44-9A3F039DCFDD}"/>
+    <hyperlink ref="G16" r:id="rId5" display="https://open.spotify.com/episode/6Rljo1PtpUiz0N779Muyp0" xr:uid="{174DB1DB-772B-43EC-AFB0-0428427A70E8}"/>
+    <hyperlink ref="G14" r:id="rId6" xr:uid="{13FFDDB7-34C5-44D7-8D29-9A080650B367}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>